<commit_message>
entrega: fotografia por rodada fica fora do git; data/out leva so o resultado oficial
Decisao do PO (opcao A): a caixa leva o resultado OFICIAL de data/out (planilha xlsx+csv, auditoria.jsonl, fila, resumo, painel, banco); as fotografias auditoria_rodada_<timestamp>.jsonl ficam so na maquina de quem roda (188 delas, agora ignoradas pelo git).

- .gitignore: data/out/auditoria_rodada_*.jsonl.
- README 5 e 7.2: bloco de saida citado = rodada real em diretorio limpo; em producao a pasta de resultados fica FORA do repositorio (mesma razao do .env: guarda dado real de cliente).
- data/out regenerado pelo comando unico: 21 artefatos, 7 aprovados, 11 revisao, 2 rejeitados, 1 duplicado, 7 linhas - identico ao declarado no README.
- Verificador: 6/6 PASSOU (exit 0).
</commit_message>
<xml_diff>
--- a/data/out/controle_financeiro.xlsx
+++ b/data/out/controle_financeiro.xlsx
@@ -521,7 +521,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-19T13:34:46-03:00</t>
+          <t>2026-09-22T07:50:08-03:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -612,7 +612,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-19T13:34:46-03:00</t>
+          <t>2026-09-22T07:50:08-03:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -703,7 +703,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-19T13:34:46-03:00</t>
+          <t>2026-09-22T07:50:08-03:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -789,7 +789,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-19T13:34:46-03:00</t>
+          <t>2026-09-22T07:50:08-03:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -880,7 +880,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-19T13:34:46-03:00</t>
+          <t>2026-09-22T07:50:08-03:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -966,7 +966,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-19T13:34:46-03:00</t>
+          <t>2026-09-22T07:50:08-03:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1057,7 +1057,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-19T13:34:46-03:00</t>
+          <t>2026-09-22T07:50:08-03:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">

</xml_diff>